<commit_message>
Player turn, tile targeting, turn order
</commit_message>
<xml_diff>
--- a/docs/CTRBLXAI_Development_Roadmap.xlsx
+++ b/docs/CTRBLXAI_Development_Roadmap.xlsx
@@ -431,26 +431,6 @@
 </a:theme>
 </file>
 
-<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
-<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="1" width="350" row="0">
-    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </wetp:taskpane>
-</wetp:taskpanes>
-</file>
-
-<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
-<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{656C07E2-B43E-4AED-A01D-BAF0B393F7F0}">
-  <we:reference id="WA200010611" version="1.0.10036.0" store="en-us" storeType="OMEX"/>
-  <we:alternateReferences/>
-  <we:properties>
-    <we:property name="Office.AutoShowTaskpaneWithDocument" value="true"/>
-  </we:properties>
-  <we:bindings/>
-  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-</we:webextension>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -546,7 +526,17 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>⬜ Not started</t>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -1252,7 +1242,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1254,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1266,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -1288,7 +1278,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -1300,7 +1290,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -1312,7 +1302,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -1324,7 +1314,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -1336,7 +1326,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1338,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -1360,7 +1350,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -1372,7 +1362,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>⏭️</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Deferred — no forced displacement system yet</t>
         </is>
       </c>
     </row>
@@ -1384,7 +1379,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
silce 3 completed. persistent hp/mp planned. rarity rules and tables documented.
</commit_message>
<xml_diff>
--- a/docs/CTRBLXAI_Development_Roadmap.xlsx
+++ b/docs/CTRBLXAI_Development_Roadmap.xlsx
@@ -16,6 +16,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice 5 - Procedural Maps" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice 6 - Content Expansion" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How To Use" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slice 7 - Visual Polish" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -437,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -627,6 +628,274 @@
       <c r="D7" t="inlineStr">
         <is>
           <t>⬜ Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Visual Polish</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Visual/audio pass: terrain, animations, VFX, UI, camera, sound</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>⬜ Not Started</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Goal:</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Make the game look and feel good — terrain materials, props, lighting, animations, UI polish, camera.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Done When:</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>A new player watches 30 seconds of gameplay and it looks like a real game, not a prototype.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Terrain tiles have distinct materials per type (grass, stone, sand, water, etc.)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Elevation visually reads clearly (cliff faces, ramps, height layers)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Each biome has a unique visual palette and props</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Map props/objects placed (trees, rocks, buildings, fences)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Lighting per biome (warm plains, cold highlands, dark caves)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Unit models distinct per weapon archetype or role</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Attack animations (swing, thrust, cast, shoot)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Skill VFX (fire burst, heal glow, poison cloud, etc.)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Status effect visual indicators on units</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CT timeline bar UI (Mana Khemia style, top of screen)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Skill Card selection UI polished</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Damage/healing numbers styled (floating, color-coded)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Camera system (follow active unit, smooth transitions)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Menu/loadout UI visual design</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Sound effects (hit, heal, status apply, UI clicks)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Music per biome or battle phase</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>⬜</t>
         </is>
       </c>
     </row>
@@ -1770,7 +2039,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="72" customWidth="1" min="1" max="1"/>
@@ -1998,6 +2267,114 @@
           <t>⬜</t>
         </is>
       </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>--- Persistent HP/MP (bundled into Slice 4) ---</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>UnitSchema accepts persistent HP/MP instead of defaulting to full</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Pass currentHp/currentMp from save state</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>MP Regen system: accumulator + CT-based tick</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>GameConstants + BattleCoordinator</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Battle-end: persist final HP/MP + apply 35% recovery</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Main.server.lua hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Battle-start: load persistent HP/MP from save state</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Main.server.lua</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>KO units get zero recovery, flagged in save</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Deployment UI shows current HP/MP before battle</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
slice 4 completion doc updates
</commit_message>
<xml_diff>
--- a/docs/CTRBLXAI_Development_Roadmap.xlsx
+++ b/docs/CTRBLXAI_Development_Roadmap.xlsx
@@ -1993,7 +1993,6 @@
           <t>After returning from battle, the player can use the Guild Base to recruit and manage units, access services, improve facilities, select activities, purchase or earn progression items, and prepare for future battles.</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2006,13 +2005,8 @@
           <t>Guild Base hub is functional: recruitment, merchants, services, quests, dispatch, explore all operational with authoritative rules. All acquisitions persist through Slice 4 APIs.</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr"/>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -2041,7 +2035,6 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2054,7 +2047,6 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2067,7 +2059,6 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2097,7 +2088,6 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2144,7 +2134,6 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2157,7 +2146,6 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2170,7 +2158,6 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2183,7 +2170,6 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2230,7 +2216,6 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2243,7 +2228,6 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2256,7 +2240,6 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2269,7 +2252,6 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2282,21 +2264,14 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr"/>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
           <t>═══ ACQUIRABLE CONTENT ═══</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2360,7 +2335,6 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2373,7 +2347,6 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2392,19 +2365,13 @@
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr"/>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
-    </row>
+    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
           <t>═══ ACQUISITION SOURCE BOUNDARY ═══</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2468,21 +2435,14 @@
           <t>RULE</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr"/>
-      <c r="B37" t="inlineStr"/>
-      <c r="C37" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="37"/>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
           <t>═══ PERSISTENCE RULE ═══</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr"/>
-      <c r="C38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2495,7 +2455,6 @@
           <t>RULE</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2508,7 +2467,6 @@
           <t>RULE</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2521,21 +2479,14 @@
           <t>RULE</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr"/>
-      <c r="B42" t="inlineStr"/>
-      <c r="C42" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="42"/>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
           <t>═══ EXISTING AUTHORITATIVE RULES IN DB ═══</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr"/>
-      <c r="C43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2690,19 +2641,13 @@
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" t="inlineStr"/>
-      <c r="B53" t="inlineStr"/>
-      <c r="C53" t="inlineStr"/>
-    </row>
+    <row r="53"/>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
           <t>═══ SPECIFIC VALUES NOT YET AUTHORED ═══</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr"/>
-      <c r="C54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2732,7 +2677,6 @@
           <t>UNDEFINED</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2745,7 +2689,6 @@
           <t>UNDEFINED</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2775,7 +2718,6 @@
           <t>UNDEFINED</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2805,7 +2747,6 @@
           <t>UNDEFINED</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2835,7 +2776,6 @@
           <t>UNDEFINED</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2871,19 +2811,13 @@
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" t="inlineStr"/>
-      <c r="B66" t="inlineStr"/>
-      <c r="C66" t="inlineStr"/>
-    </row>
+    <row r="66"/>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
           <t>═══ SLICE OWNERSHIP ═══</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr"/>
-      <c r="C67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2896,7 +2830,6 @@
           <t>Guild Base framework, merchants, purchases, recruitment, quest/activity rewards, Doctrine/Skill Card/Augment Card acquisition workflows, Tavern, Blacksmith, facility, Guild progression, management workflows, service costs, unlocks, battle-prep transition</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2909,7 +2842,6 @@
           <t>Inventory ownership, roster ownership, equipment/loadout state, equip/unequip, save/load, adding acquired items to persistent inventory, restoring after rejoin, battle reward commitment, minimal functional Loadout Hub</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2922,7 +2854,6 @@
           <t>Content catalogs: equipment, consumables, Doctrines, Skill Cards, Augment Cards</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2935,7 +2866,6 @@
           <t>Guild Base visual presentation, merchant-screen layout, reward/acquisition presentation, item/Doctrine/Skill Card/Augment Card visual components, icons, portraits, rarity, themes, animations, VFX, responsive layout, UI sound</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2948,21 +2878,14 @@
           <t>Must not duplicate Slice 4 persistence, redefine Slice 6 content, or build Slice 7 presentation</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr"/>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr"/>
-      <c r="B73" t="inlineStr"/>
-      <c r="C73" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="73"/>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
           <t>═══ BLOCKERS AND STATUS ═══</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr"/>
-      <c r="C74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3009,7 +2932,6 @@
           <t>DEP</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -3022,13 +2944,8 @@
           <t>DEP</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr"/>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr"/>
-      <c r="B79" t="inlineStr"/>
-      <c r="C79" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="79"/>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
@@ -3040,7 +2957,6 @@
           <t>⬜ Not Started</t>
         </is>
       </c>
-      <c r="C80" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5010,6 +4926,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -5035,7 +4952,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5047,7 +4964,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5059,7 +4976,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5071,7 +4988,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5083,7 +5000,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5095,7 +5012,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5107,7 +5024,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5119,7 +5036,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5131,7 +5048,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5143,7 +5060,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5155,7 +5072,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5167,10 +5084,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
@@ -5186,7 +5104,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -5203,7 +5121,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -5220,7 +5138,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -5237,7 +5155,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -5254,10 +5172,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
@@ -5265,6 +5184,7 @@
         </is>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
@@ -5277,6 +5197,7 @@
         </is>
       </c>
     </row>
+    <row r="28"/>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
@@ -5292,7 +5213,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -5309,7 +5230,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5321,7 +5242,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -5338,7 +5259,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -5355,7 +5276,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5367,7 +5288,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -5384,7 +5305,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -5401,7 +5322,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5413,7 +5334,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5425,10 +5346,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="40"/>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
@@ -5444,7 +5366,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -5461,7 +5383,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -5478,7 +5400,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -5495,7 +5417,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SLICE 7</t>
+          <t>⏭️ Slice 7</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -5504,6 +5426,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
@@ -5519,7 +5442,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -5536,7 +5459,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5548,7 +5471,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>SLICE 7</t>
+          <t>⏭️ Slice 7</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -5557,6 +5480,7 @@
         </is>
       </c>
     </row>
+    <row r="51"/>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
@@ -5572,7 +5496,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -5589,7 +5513,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5601,7 +5525,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>SLICE 7</t>
+          <t>⏭️ Slice 7</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -5610,6 +5534,7 @@
         </is>
       </c>
     </row>
+    <row r="56"/>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
@@ -5625,7 +5550,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -5642,7 +5567,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5654,7 +5579,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -5671,7 +5596,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -5688,7 +5613,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5700,7 +5625,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>SLICE 7</t>
+          <t>⏭️ Slice 7</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -5709,6 +5634,7 @@
         </is>
       </c>
     </row>
+    <row r="64"/>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
@@ -5724,7 +5650,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -5741,7 +5667,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5753,7 +5679,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>SLICE 7</t>
+          <t>⏭️ Slice 7</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -5762,6 +5688,7 @@
         </is>
       </c>
     </row>
+    <row r="69"/>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
@@ -5777,7 +5704,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -5794,7 +5721,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>⏭️ Slice 7</t>
         </is>
       </c>
     </row>
@@ -5823,7 +5750,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>⏭️ Slice 7</t>
         </is>
       </c>
     </row>
@@ -5835,10 +5762,11 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
+          <t>⏭️ Slice 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="76"/>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
@@ -5871,7 +5799,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5883,7 +5811,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5895,7 +5823,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5907,7 +5835,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5919,7 +5847,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5859,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5943,7 +5871,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5955,7 +5883,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5967,7 +5895,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -5979,7 +5907,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>⏭️ Slice 7</t>
         </is>
       </c>
     </row>
@@ -5991,7 +5919,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>⏭️ Slice 7</t>
         </is>
       </c>
     </row>
@@ -6003,7 +5931,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -6015,10 +5943,11 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>⬜</t>
-        </is>
-      </c>
-    </row>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="92"/>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
@@ -6041,7 +5970,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -6053,7 +5982,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -6065,7 +5994,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -6077,7 +6006,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -6089,7 +6018,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -6101,7 +6030,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -6113,7 +6042,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -6125,7 +6054,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -6137,7 +6066,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -6149,7 +6078,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -6161,7 +6090,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -6180,7 +6109,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>✅</t>
         </is>
       </c>
     </row>
@@ -6192,7 +6121,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>⏭️ Slice 7</t>
         </is>
       </c>
     </row>
@@ -6204,7 +6133,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>⏭️ Slice 7</t>
         </is>
       </c>
     </row>
@@ -6220,6 +6149,7 @@
         </is>
       </c>
     </row>
+    <row r="111"/>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
@@ -6295,18 +6225,20 @@
         </is>
       </c>
     </row>
+    <row r="117"/>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>VERDICT: READY WITH BLOCKERS</t>
+          <t>VERDICT: SLICE 4 FUNCTIONALLY COMPLETE (2026-08-31)</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Reward transaction work may continue only after Item Level decision is approved.</t>
-        </is>
-      </c>
-    </row>
+          <t>Visual presentation deferred to Slice 7. Map Level placeholder awaits Slice 5. Doctrine Break/Augment attachment unassigned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119"/>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
@@ -6418,7 +6350,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>⬜ In Progress</t>
+          <t>✅ Complete (2026-08-31)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Implement race data and passive effects
- Added RaceData.lua to define various races, their starting stats, growth rates, and passive abilities.
- Introduced RacePassiveService.lua to centralize race passive effect calculations, including damage modifiers, MP cost adjustments, and movement range penalties.
- Updated UnitInspectorPanel.client.lua to integrate new theme settings and improve UI layout for displaying unit stats and traits.
- Enhanced the rendering of traits in the inspector panel, including active buffs and debuffs, race passives, and doctrines.
</commit_message>
<xml_diff>
--- a/docs/CTRBLXAI_Development_Roadmap.xlsx
+++ b/docs/CTRBLXAI_Development_Roadmap.xlsx
@@ -788,7 +788,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C108"/>
+  <dimension ref="A1:C174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1967,6 +1967,787 @@
           <t>🔄 In Progress — Stage 1 Desktop Checkpoint: e8dcc977</t>
         </is>
       </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>═══ STAGE 2A: ROSTER AND UNIT LOADOUT PRESENTATION ═══</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr"/>
+      <c r="C110" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr"/>
+      <c r="B111" t="inlineStr"/>
+      <c r="C111" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Goal:</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Three-tab Loadout Hub (Info / Equipment / Skills) with persistent unit header, responsive layout, Theme-consistent presentation. Full spec in DB: loadout_ui_spec (59 rules).</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr"/>
+      <c r="B113" t="inlineStr"/>
+      <c r="C113" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>--- Shared Navigation ---</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr"/>
+      <c r="C114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Three tabs at top: INFO | EQUIPMENT | SKILLS</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Aligned beside Roblox system controls</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Persistent unit header: portrait, name, level, race, doctrine, 3x2 stat grid</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Upper-right on all tabs, compact</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Previous/next unit controls + tap-portrait unit selector</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Management selection only — no battle state change</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Unit switching preserves tab, refreshes all data, clears stale selections</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Pending-change guard on unit switch (confirm/cancel/discard)</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr"/>
+      <c r="B120" t="inlineStr"/>
+      <c r="C120" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>--- Info Tab ---</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr"/>
+      <c r="C121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Primary stats with breakdown (base, allocation, equipment, doctrine)</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>STR INT DEX / AGI VIT LUK</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Stat allocation controls (only in Info)</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>No respec — Slice 7 must not implement</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Secondary stats display with authoritative breakdown on select</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>No Critical Rate, Critical Damage, Evasion</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Race info: icon, name, growth rates, Race Perk, Race Drawback</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Separate labels from Unit Perk/Drawback</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Generated unit traits: one Perk, one Drawback</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Doctrine summary (display-only, managed from Equipment)</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Unit records (only when authoritative data exists)</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr"/>
+      <c r="B129" t="inlineStr"/>
+      <c r="C129" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>--- Equipment Tab ---</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr"/>
+      <c r="C130" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Inventory grid (left) + loadout (right) layout</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Square item cards, scrollable</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Complete loadout: MainHand, OffHand, Head, Torso, Arms, Legs, Accessory, 6 Consumable slots, Doctrine</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Off-Hand disabled when 2H equipped</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Consumable slots 1-3 usable, 4-6 visible locked with explanation</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Doctrine: mandatory, swap-only, cannot be empty or unequipped</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Item-type filters, rarity filter, sorting, search</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Item selection → comparison → equip/replace/swap transaction</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>BP never shown in any player-facing UI</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>RULE</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr"/>
+      <c r="B139" t="inlineStr"/>
+      <c r="C139" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>--- Equipment Comparison ---</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr"/>
+      <c r="C140" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Current vs selected, only changed values</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Colors reflect gameplay consequence, not just math sign</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Authoritative before-and-after from Slice 4 — no independent calculation</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>RULE</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr"/>
+      <c r="B143" t="inlineStr"/>
+      <c r="C143" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>--- Doctrine Comparison ---</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr"/>
+      <c r="C144" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Swap Doctrine only (no Unequip). Warn if Doctrine Skill in Slot 1 affected</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr"/>
+      <c r="B146" t="inlineStr"/>
+      <c r="C146" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>--- Skills Tab ---</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr"/>
+      <c r="C147" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Five Skill rows: slot, icon, name, effect, MP, RT, 2 augment slots each</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Slot 1: Doctrine Skill (3 choices from doctrine, player selects one)</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Cannot accept normal Skill Card</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Slots 2-4: Skill Cards with 2 Augment slots each</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Slot 5: visible locked — 'Locked by First Race Evolution'</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Skill Card + Augment Card inventory with subtabs, stacking</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Skill Card details: full authoritative fields, formulas displayed not evaluated</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Augment Card details: compatibility from functional system, modified costs shown</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Filters: type, tags, element, compatibility</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr"/>
+      <c r="B156" t="inlineStr"/>
+      <c r="C156" t="inlineStr"/>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>--- Interaction ---</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr"/>
+      <c r="C157" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Desktop: drag-and-drop + click-to-select for Skills/Augments</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Mobile: tap → highlight destinations → tap destination → preview → confirm</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Drag must not be only method</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Pending change preview before all commits</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr"/>
+      <c r="B161" t="inlineStr"/>
+      <c r="C161" t="inlineStr"/>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>--- Responsive ---</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr"/>
+      <c r="C162" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Mobile-first layout, desktop expanded</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Roblox controls unobstructed, tabs at top, no full rebuild on switch</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>RULE</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr"/>
+      <c r="B165" t="inlineStr"/>
+      <c r="C165" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>--- Loadout Presentation Completion Gate ---</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr"/>
+      <c r="C166" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Three tabs consistent, Roblox controls clear, unit switching works</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr"/>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Info: accurate stats, allocation only in Info, no nonexistent stats</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr"/>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Equipment: square cards, no BP, accurate comparison, doctrine swap-only</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr"/>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Skills: doctrine skill slot 1, skill cards 2-4, locked slot 5, augment slots</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr"/>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Mobile tap-based management works, desktop drag works</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr"/>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Pending changes cannot be silently lost</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr"/>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>No Slice 7 interface calculates authoritative gameplay values</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>RULE</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr"/>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Save and reload preserve all committed loadout changes</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2006,7 +2787,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -2265,7 +3045,6 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
@@ -2365,7 +3144,6 @@
         </is>
       </c>
     </row>
-    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
@@ -2436,7 +3214,6 @@
         </is>
       </c>
     </row>
-    <row r="37"/>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
@@ -2480,7 +3257,6 @@
         </is>
       </c>
     </row>
-    <row r="42"/>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
@@ -2641,7 +3417,6 @@
         </is>
       </c>
     </row>
-    <row r="53"/>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
@@ -2811,7 +3586,6 @@
         </is>
       </c>
     </row>
-    <row r="66"/>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
@@ -2879,7 +3653,6 @@
         </is>
       </c>
     </row>
-    <row r="73"/>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
@@ -2945,7 +3718,6 @@
         </is>
       </c>
     </row>
-    <row r="79"/>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
@@ -4926,7 +5698,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -5088,7 +5859,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
@@ -5176,7 +5946,6 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
@@ -5184,7 +5953,6 @@
         </is>
       </c>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
@@ -5197,7 +5965,6 @@
         </is>
       </c>
     </row>
-    <row r="28"/>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
@@ -5350,7 +6117,6 @@
         </is>
       </c>
     </row>
-    <row r="40"/>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
@@ -5426,7 +6192,6 @@
         </is>
       </c>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
@@ -5480,7 +6245,6 @@
         </is>
       </c>
     </row>
-    <row r="51"/>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
@@ -5534,7 +6298,6 @@
         </is>
       </c>
     </row>
-    <row r="56"/>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
@@ -5634,7 +6397,6 @@
         </is>
       </c>
     </row>
-    <row r="64"/>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
@@ -5688,7 +6450,6 @@
         </is>
       </c>
     </row>
-    <row r="69"/>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
@@ -5766,7 +6527,6 @@
         </is>
       </c>
     </row>
-    <row r="76"/>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
@@ -5947,7 +6707,6 @@
         </is>
       </c>
     </row>
-    <row r="92"/>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
@@ -6149,7 +6908,6 @@
         </is>
       </c>
     </row>
-    <row r="111"/>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
@@ -6225,7 +6983,6 @@
         </is>
       </c>
     </row>
-    <row r="117"/>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
@@ -6238,7 +6995,6 @@
         </is>
       </c>
     </row>
-    <row r="119"/>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Slice 3 Foundation: 36 new status defs, action blocking, turn skip, Petrify DR, element system with interactions/triggers, LoS unit blocking, Frozen removed from hard CC
</commit_message>
<xml_diff>
--- a/docs/CTRBLXAI_Development_Roadmap.xlsx
+++ b/docs/CTRBLXAI_Development_Roadmap.xlsx
@@ -589,7 +589,17 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>⬜ Not started</t>
+          <t>✅ Done</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
@@ -649,7 +659,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>🔄 In Progress — Stage 1 Desktop Checkpoint Verified</t>
+          <t>🔄 In Progress — Stage 1 Complete, Stage 2 (Battle UI + Loadout) In Progress</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -788,7 +798,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C174"/>
+  <dimension ref="A1:C186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -815,6 +825,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -948,7 +959,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>🔄</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>BattleHUD.lua expanded from 37KB to 66KB; UpdateTimeline exists</t>
         </is>
       </c>
     </row>
@@ -960,7 +976,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>🔄</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>BattleHUD.ShowSkillList/ShowSkillDetail exist</t>
         </is>
       </c>
     </row>
@@ -972,7 +993,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>🔄</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>showDamageText/showFloatingText exist in BattleVisualClient</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1027,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>🔄</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>LoadoutScreen.lua (76KB) created; LoadoutController.client.lua exists</t>
         </is>
       </c>
     </row>
@@ -1029,6 +1060,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
@@ -1036,6 +1068,7 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
@@ -1281,6 +1314,7 @@
         </is>
       </c>
     </row>
+    <row r="44"/>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
@@ -1363,6 +1397,7 @@
         </is>
       </c>
     </row>
+    <row r="51"/>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
@@ -1404,6 +1439,7 @@
         </is>
       </c>
     </row>
+    <row r="55"/>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
@@ -1500,6 +1536,7 @@
         </is>
       </c>
     </row>
+    <row r="64"/>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
@@ -1563,6 +1600,7 @@
         </is>
       </c>
     </row>
+    <row r="69"/>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
@@ -1570,6 +1608,7 @@
         </is>
       </c>
     </row>
+    <row r="71"/>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
@@ -1661,6 +1700,7 @@
         </is>
       </c>
     </row>
+    <row r="80"/>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
@@ -1836,6 +1876,7 @@
         </is>
       </c>
     </row>
+    <row r="96"/>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
@@ -1853,6 +1894,7 @@
         </is>
       </c>
     </row>
+    <row r="98"/>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
@@ -1968,20 +2010,15 @@
         </is>
       </c>
     </row>
+    <row r="109"/>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
           <t>═══ STAGE 2A: ROSTER AND UNIT LOADOUT PRESENTATION ═══</t>
         </is>
       </c>
-      <c r="B110" t="inlineStr"/>
-      <c r="C110" t="inlineStr"/>
-    </row>
-    <row r="111">
-      <c r="A111" t="inlineStr"/>
-      <c r="B111" t="inlineStr"/>
-      <c r="C111" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="111"/>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
@@ -1993,21 +2030,14 @@
           <t>Three-tab Loadout Hub (Info / Equipment / Skills) with persistent unit header, responsive layout, Theme-consistent presentation. Full spec in DB: loadout_ui_spec (59 rules).</t>
         </is>
       </c>
-      <c r="C112" t="inlineStr"/>
-    </row>
-    <row r="113">
-      <c r="A113" t="inlineStr"/>
-      <c r="B113" t="inlineStr"/>
-      <c r="C113" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="113"/>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
           <t>--- Shared Navigation ---</t>
         </is>
       </c>
-      <c r="B114" t="inlineStr"/>
-      <c r="C114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -2017,12 +2047,12 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>🔄</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Aligned beside Roblox system controls</t>
+          <t>LoadoutScreen.lua implements tab structure</t>
         </is>
       </c>
     </row>
@@ -2034,12 +2064,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>🔄</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Upper-right on all tabs, compact</t>
+          <t>LoadoutScreen.lua implements header</t>
         </is>
       </c>
     </row>
@@ -2051,12 +2081,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>🔄</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Management selection only — no battle state change</t>
+          <t>LoadoutScreen.lua implements unit switching</t>
         </is>
       </c>
     </row>
@@ -2071,7 +2101,6 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -2084,21 +2113,14 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C119" t="inlineStr"/>
-    </row>
-    <row r="120">
-      <c r="A120" t="inlineStr"/>
-      <c r="B120" t="inlineStr"/>
-      <c r="C120" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="120"/>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
           <t>--- Info Tab ---</t>
         </is>
       </c>
-      <c r="B121" t="inlineStr"/>
-      <c r="C121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -2179,7 +2201,6 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -2192,7 +2213,6 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -2205,21 +2225,14 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C128" t="inlineStr"/>
-    </row>
-    <row r="129">
-      <c r="A129" t="inlineStr"/>
-      <c r="B129" t="inlineStr"/>
-      <c r="C129" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="129"/>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
           <t>--- Equipment Tab ---</t>
         </is>
       </c>
-      <c r="B130" t="inlineStr"/>
-      <c r="C130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -2229,12 +2242,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>⬜</t>
+          <t>🔄</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Square item cards, scrollable</t>
+          <t>LoadoutScreen.lua implements inventory grid</t>
         </is>
       </c>
     </row>
@@ -2246,10 +2259,14 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="C132" t="inlineStr"/>
+          <t>🔄</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>LoadoutScreen.lua implements equipment slots</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -2262,7 +2279,6 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -2275,7 +2291,6 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -2288,7 +2303,6 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -2298,10 +2312,14 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="C136" t="inlineStr"/>
+          <t>🔄</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>LoadoutScreen.lua implements filters</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -2311,10 +2329,14 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>⬜</t>
-        </is>
-      </c>
-      <c r="C137" t="inlineStr"/>
+          <t>🔄</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>LoadoutScreen.BuildItemDetail exists</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -2333,19 +2355,13 @@
         </is>
       </c>
     </row>
-    <row r="139">
-      <c r="A139" t="inlineStr"/>
-      <c r="B139" t="inlineStr"/>
-      <c r="C139" t="inlineStr"/>
-    </row>
+    <row r="139"/>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
           <t>--- Equipment Comparison ---</t>
         </is>
       </c>
-      <c r="B140" t="inlineStr"/>
-      <c r="C140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -2381,19 +2397,13 @@
         </is>
       </c>
     </row>
-    <row r="143">
-      <c r="A143" t="inlineStr"/>
-      <c r="B143" t="inlineStr"/>
-      <c r="C143" t="inlineStr"/>
-    </row>
+    <row r="143"/>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
           <t>--- Doctrine Comparison ---</t>
         </is>
       </c>
-      <c r="B144" t="inlineStr"/>
-      <c r="C144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -2406,21 +2416,14 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C145" t="inlineStr"/>
-    </row>
-    <row r="146">
-      <c r="A146" t="inlineStr"/>
-      <c r="B146" t="inlineStr"/>
-      <c r="C146" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="146"/>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
           <t>--- Skills Tab ---</t>
         </is>
       </c>
-      <c r="B147" t="inlineStr"/>
-      <c r="C147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -2433,7 +2436,6 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -2463,7 +2465,6 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -2476,7 +2477,6 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -2489,7 +2489,6 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -2502,7 +2501,6 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -2515,7 +2513,6 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -2528,21 +2525,14 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C155" t="inlineStr"/>
-    </row>
-    <row r="156">
-      <c r="A156" t="inlineStr"/>
-      <c r="B156" t="inlineStr"/>
-      <c r="C156" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="156"/>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
           <t>--- Interaction ---</t>
         </is>
       </c>
-      <c r="B157" t="inlineStr"/>
-      <c r="C157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -2555,7 +2545,6 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -2585,21 +2574,14 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C160" t="inlineStr"/>
-    </row>
-    <row r="161">
-      <c r="A161" t="inlineStr"/>
-      <c r="B161" t="inlineStr"/>
-      <c r="C161" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="161"/>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
           <t>--- Responsive ---</t>
         </is>
       </c>
-      <c r="B162" t="inlineStr"/>
-      <c r="C162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -2612,7 +2594,6 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -2631,19 +2612,13 @@
         </is>
       </c>
     </row>
-    <row r="165">
-      <c r="A165" t="inlineStr"/>
-      <c r="B165" t="inlineStr"/>
-      <c r="C165" t="inlineStr"/>
-    </row>
+    <row r="165"/>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
           <t>--- Loadout Presentation Completion Gate ---</t>
         </is>
       </c>
-      <c r="B166" t="inlineStr"/>
-      <c r="C166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -2656,7 +2631,6 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -2669,7 +2643,6 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -2682,7 +2655,6 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -2695,7 +2667,6 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -2708,7 +2679,6 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -2721,7 +2691,6 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -2734,7 +2703,6 @@
           <t>RULE</t>
         </is>
       </c>
-      <c r="C173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -2747,7 +2715,149 @@
           <t>⬜</t>
         </is>
       </c>
-      <c r="C174" t="inlineStr"/>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>═══ STAGE 2B: BATTLE HUD EXPANSION (tracked post-audit) ═══</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr"/>
+      <c r="C176" t="inlineStr"/>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr"/>
+      <c r="B177" t="inlineStr"/>
+      <c r="C177" t="inlineStr"/>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>BattleHUD.lua expanded to 66KB (from 37KB baseline)</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>🔄</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Major expansion: actor/target cards, skill list, damage preview, tile info, battle log, phase display, tooltips, confirm bar</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Theme.lua expanded to 20KB (from 7KB baseline)</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>🔄</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Expanded color palette, rarity colors, spacing tokens</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>BattleVisualClient.lua expanded to 83KB (from 62KB baseline)</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>🔄</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>LoadoutScreen integration, expanded event handlers</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>UnitInspectorPanel.lua at 24KB</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>🔄</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>3-tab inspector (Stats/Equipment/Skills)</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr"/>
+      <c r="B182" t="inlineStr"/>
+      <c r="C182" t="inlineStr"/>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>--- New Modules Created ---</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr"/>
+      <c r="C183" t="inlineStr"/>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>LoadoutScreen.lua (76KB) — full loadout UI implementation</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>🔄</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Slice 7 Stage 2A</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>MockLoadoutData.lua (25KB) — test data for loadout development</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>🔄</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Development aid</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>LoadoutController.client.lua (2KB) — entry point, L key toggle</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5185,7 +5295,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="72" customWidth="1" min="1" max="1"/>
@@ -5652,6 +5762,753 @@
       <c r="B33" t="inlineStr">
         <is>
           <t>Completed 2026-08-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>═══ SLICE 3 FOUNDATION EXPANSION (post-completion) ═══</t>
+        </is>
+      </c>
+    </row>
+    <row r="36"/>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>--- Phase 1: Status Definitions ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>GameConstants.STATUSES expanded from 4 → 36 entries (all DB statuses)</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Includes Sleep, Silence, Stun, Petrify, Haste, Wet, Frozen, etc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39"/>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>--- Phase 2: StatusService Expansion ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>StatusService.IsActionBlocked exists (Silence→skills, Disarmed→attack, Pinned→move)</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>🔄</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Sleep/Stun/Petrify blocking implemented; Disarmed/Pinned referenced but not fully tested</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Turn-skipping statuses (Sleep, Petrify, Stun) in BattleCoordinator</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Needs verification</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Hard CC removes Guard on application</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Sleep/Petrify should remove Guard — needs verification</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Status tick behaviors beyond DoT (Haste RT mod, Regeneration, Weakened, etc.)</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>36 statuses defined; most tick behaviors not yet in StatusService runtime</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Reapplication rules per status</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>DB defines per-status reapplication; StatusService may not enforce all</t>
+        </is>
+      </c>
+    </row>
+    <row r="46"/>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>--- Phase 3: Element System ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Element tag extraction in CombatResolver</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>🔄</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Element extraction logic exists; full interaction chain incomplete</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Element→status triggers (Fire→Burn, Water→Wet, Ice+Wet→Frozen)</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Element weakness/resistance multipliers</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Depends on Phase 5 race tags for full effect</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Healing element interactions (Holy vs Undead)</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Depends on Phase 5 Undead tag</t>
+        </is>
+      </c>
+    </row>
+    <row r="52"/>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>--- Phase 4: Status Immunity Framework ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Immunity check before status application</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>No IsImmune check in StatusService.ApplyStatus</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Race-tag immunities registered (Undead, Mechanical)</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Debuff Resistance stat functional (VIT-based)</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Still defaults to 1.0 in code</t>
+        </is>
+      </c>
+    </row>
+    <row r="57"/>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>--- Phase 5: Race Tag Functional Effects ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Race tags stored on unit at creation</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>RaceData has tags; UnitSchema doesn't copy to unit.tags</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Undead: healing reversal, Holy×2, immunities</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Mechanical: WT+15%, immunities, Wet doubled</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Amphibious: water movement, Drowning immunity</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Blocked — no water tiles in combat</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Flying: permanent Flight</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Blocked — Flight status not fully implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Giant: melee elevation range, knockback</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>⬜</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Giant tag added to DB (2026-09-04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65"/>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>--- Phase 6: Race Passive Evaluation ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>RacePassiveService.lua created with 8 query functions</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>6.4KB — integrated into CombatResolver, CommandService, TargetingService, EquipmentService</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Orc Bloodlust (below 50% HP → +15% damage)</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>In RacePassiveService.GetDamageDealtModifier</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Dwarf Stout Resilience (physical DR -10%, Move -1)</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>DR in GetDamageReceivedModifier, Move in GetMovementRangeModifier</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Fairy Fae Grace (AOE DR -25%, STR -15%)</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>DR in GetDamageReceivedModifier, STR in GetStatModifiers</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Golem Fortified Frame (Guard +20%, Move -1)</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Guard in GetGuardMitigationBonus, Move in GetMovementRangeModifier</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Zombie Undying (Move -1)</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>🔄</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Movement penalty applied; revive NOT implemented (no revive system)</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Elf Elven Focus (MP Cost -20%)</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>In RacePassiveService.GetMpCostModifier</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Elf Jump +1</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>NOT applied — ComputeDerivedStats uses formula only, no race bonus</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Goblin Basic Attack applies Poison</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>🔄</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>GetBasicAttackStatus returns 'Poison'; needs CombatResolver integration verification</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Elemental Spirit elemental damage +30%/-30%</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>In GetDamageDealtModifier and GetDamageReceivedModifier</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Lich Arcane Corruption (Light damage received +50%)</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>In GetDamageReceivedModifier</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Shadow Umbral Veil (elemental DR +10%; Hide pending)</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>🔄</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>DR applied; Hide-on-hit NOT implemented (no Hide status)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Titan CanEquip2HAsWith1H</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>In RacePassiveService and EquipmentService</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Vampire lifesteal (15%/5%)</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>NOT implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Human Adaptability (EXP +10%, +1 stat/3 levels)</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Blocked — no leveling/EXP system</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Android Push→Pull</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Blocked — DisplacementService needs Pull mechanic</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Mermaid Tidecaller (water tile bonuses)</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Blocked — no water tiles in combat</t>
+        </is>
+      </c>
+    </row>
+    <row r="84"/>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>--- Phase 7: Content Registry Bridge ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>SkillData.lua generated (89 skills from DB)</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>118KB data file</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>AugmentData.lua generated (102 augments from DB)</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>91KB data file</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>DoctrineData.lua generated (32 doctrines from DB)</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>33KB data file</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Registry.lua facade (GetSkill/GetAugment/GetDoctrine)</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Battle systems consume Content Registry instead of hardcoded GameConstants.SKILLS</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>CommandService/CombatResolver still use 6 hardcoded skills</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Formula evaluator for SkillData string formulas</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>❌</t>
         </is>
       </c>
     </row>

</xml_diff>